<commit_message>
update: game mechanics; add: deda sprites and animations
</commit_message>
<xml_diff>
--- a/leaderboard.xlsx
+++ b/leaderboard.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,520 +443,320 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>auuu</t>
+          <t>auhhh</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14200</v>
+        <v>14700</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>vojislavu</t>
+          <t>auuuu</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12900</v>
+        <v>14400</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>vojislav</t>
+          <t>bash</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12700</v>
+        <v>14200</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>jksdaouihasduhi</t>
+          <t>a</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12500</v>
+        <v>14100</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>abv</t>
+          <t>nije rekord</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12300</v>
+        <v>14100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>aaaa</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12100</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>voki</t>
+          <t>zeznuto</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12100</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>vojislav voki</t>
+          <t>aaa kurac</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12100</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>vojimir</t>
+          <t>aaaa</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>12100</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>Vojislav</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12000</v>
+        <v>12400</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>jaoo bas jesam</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12000</v>
+        <v>12300</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>eejejeje</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>11900</v>
+        <v>12200</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>alahu ekber</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11700</v>
+        <v>12200</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>nisaaam</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10900</v>
+        <v>12100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>kurac</t>
+          <t>tuzan sam</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10700</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>avangarda</t>
+          <t>nisaaam</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10300</v>
+        <v>11600</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>vopislav</t>
+          <t>a</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>10300</v>
+        <v>11200</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>aaaaa</t>
+          <t>nisam odvinjacio</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>10100</v>
+        <v>10400</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>kurcina</t>
+          <t>aaa</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8700</v>
+        <v>10100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>Vo jislav</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7900</v>
+        <v>10100</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>Lep dan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6200</v>
+        <v>9800</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>a</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6200</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>kurac</t>
+          <t>Vojin</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5700</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>n</t>
+          <t xml:space="preserve">Vojislav </t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4200</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>guza</t>
+          <t>a</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>Abcd</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4000</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Efgh</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>IJKL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2800</v>
+        <v>900</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>MNOP</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>RSTU</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>AAAA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Abcd</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>aaaaqqq</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>deaa</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>debeli guzon</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>debeli guzon</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>kurac</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>asdadasu9hashuad</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>aa</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add: streamlit app and requirements (#1)
* add: streamlit app and requirements
* update: streamlit app confiugration loading
* update: reqs
* update: streamlit app to include game leaderboard and gallery of images
* update: streamlit with nicer UI
* update: ispovedaonica text
* update: game mechanics; add: deda sprites and animations
</commit_message>
<xml_diff>
--- a/leaderboard.xlsx
+++ b/leaderboard.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,520 +443,320 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>auuu</t>
+          <t>auhhh</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14200</v>
+        <v>14700</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>vojislavu</t>
+          <t>auuuu</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12900</v>
+        <v>14400</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>vojislav</t>
+          <t>bash</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12700</v>
+        <v>14200</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>jksdaouihasduhi</t>
+          <t>a</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12500</v>
+        <v>14100</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>abv</t>
+          <t>nije rekord</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12300</v>
+        <v>14100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>aaaa</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12100</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>voki</t>
+          <t>zeznuto</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12100</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>vojislav voki</t>
+          <t>aaa kurac</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12100</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>vojimir</t>
+          <t>aaaa</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>12100</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>Vojislav</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12000</v>
+        <v>12400</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>jaoo bas jesam</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12000</v>
+        <v>12300</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>eejejeje</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>11900</v>
+        <v>12200</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>alahu ekber</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11700</v>
+        <v>12200</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>nisaaam</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10900</v>
+        <v>12100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>kurac</t>
+          <t>tuzan sam</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10700</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>avangarda</t>
+          <t>nisaaam</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10300</v>
+        <v>11600</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>vopislav</t>
+          <t>a</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>10300</v>
+        <v>11200</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>aaaaa</t>
+          <t>nisam odvinjacio</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>10100</v>
+        <v>10400</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>kurcina</t>
+          <t>aaa</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8700</v>
+        <v>10100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>Vo jislav</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7900</v>
+        <v>10100</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>Lep dan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6200</v>
+        <v>9800</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>a</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6200</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>kurac</t>
+          <t>Vojin</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5700</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>n</t>
+          <t xml:space="preserve">Vojislav </t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4200</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>guza</t>
+          <t>a</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>Abcd</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4000</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Efgh</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>IJKL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2800</v>
+        <v>900</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>MNOP</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>RSTU</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>AAAA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Abcd</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>aaaaqqq</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>deaa</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>debeli guzon</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>debeli guzon</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>kurac</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>asdadasu9hashuad</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>aa</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>